<commit_message>
Update raw inventory, sales, and supplier datasets
</commit_message>
<xml_diff>
--- a/data/sample/supplier_raw_data.xlsx
+++ b/data/sample/supplier_raw_data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rajar\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rajar\OneDrive\Desktop\Supply-Chain-Analytics-rajarshi\data\sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABDE22C0-0D81-475F-BD40-5C0471D7E564}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7794947F-F7C1-4904-B07A-0BB33AF87C5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4008" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4736" uniqueCount="382">
   <si>
     <t>supplier_id</t>
   </si>
@@ -1508,7 +1508,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I801"/>
+  <dimension ref="A1:I951"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.5546875" customWidth="1"/>
@@ -22348,6 +22348,3822 @@
         <v>3450</v>
       </c>
     </row>
+    <row r="802" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="C802" t="s">
+        <v>15</v>
+      </c>
+      <c r="E802" t="s">
+        <v>126</v>
+      </c>
+      <c r="F802">
+        <v>-4</v>
+      </c>
+      <c r="H802">
+        <v>3744</v>
+      </c>
+    </row>
+    <row r="803" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A803" t="s">
+        <v>29</v>
+      </c>
+      <c r="B803" t="s">
+        <v>30</v>
+      </c>
+      <c r="C803" t="s">
+        <v>36</v>
+      </c>
+      <c r="D803" t="s">
+        <v>120</v>
+      </c>
+      <c r="E803" t="s">
+        <v>97</v>
+      </c>
+      <c r="F803">
+        <v>5</v>
+      </c>
+      <c r="G803">
+        <v>4.49</v>
+      </c>
+      <c r="H803">
+        <v>3870</v>
+      </c>
+    </row>
+    <row r="804" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A804" t="s">
+        <v>17</v>
+      </c>
+      <c r="B804" t="s">
+        <v>18</v>
+      </c>
+      <c r="C804" t="s">
+        <v>19</v>
+      </c>
+      <c r="D804" t="s">
+        <v>33</v>
+      </c>
+      <c r="E804" t="s">
+        <v>114</v>
+      </c>
+      <c r="F804">
+        <v>6</v>
+      </c>
+      <c r="G804">
+        <v>2.83</v>
+      </c>
+      <c r="H804">
+        <v>1742</v>
+      </c>
+    </row>
+    <row r="805" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A805" t="s">
+        <v>17</v>
+      </c>
+      <c r="B805" t="s">
+        <v>18</v>
+      </c>
+      <c r="C805" t="s">
+        <v>15</v>
+      </c>
+      <c r="D805" t="s">
+        <v>59</v>
+      </c>
+      <c r="E805" t="s">
+        <v>59</v>
+      </c>
+      <c r="F805">
+        <v>-3</v>
+      </c>
+      <c r="G805">
+        <v>3.45</v>
+      </c>
+      <c r="H805">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="806" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A806" t="s">
+        <v>8</v>
+      </c>
+      <c r="B806" t="s">
+        <v>9</v>
+      </c>
+      <c r="C806" t="s">
+        <v>36</v>
+      </c>
+      <c r="D806" t="s">
+        <v>188</v>
+      </c>
+      <c r="E806" t="s">
+        <v>188</v>
+      </c>
+      <c r="F806">
+        <v>0</v>
+      </c>
+      <c r="G806">
+        <v>4.6100000000000003</v>
+      </c>
+      <c r="H806">
+        <v>3354</v>
+      </c>
+    </row>
+    <row r="807" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A807" t="s">
+        <v>17</v>
+      </c>
+      <c r="B807" t="s">
+        <v>18</v>
+      </c>
+      <c r="C807" t="s">
+        <v>19</v>
+      </c>
+      <c r="D807" t="s">
+        <v>83</v>
+      </c>
+      <c r="E807" t="s">
+        <v>274</v>
+      </c>
+      <c r="F807">
+        <v>4</v>
+      </c>
+      <c r="G807">
+        <v>4.51</v>
+      </c>
+      <c r="H807">
+        <v>845</v>
+      </c>
+    </row>
+    <row r="808" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A808" t="s">
+        <v>13</v>
+      </c>
+      <c r="B808" t="s">
+        <v>14</v>
+      </c>
+      <c r="C808" t="s">
+        <v>10</v>
+      </c>
+      <c r="D808" t="s">
+        <v>131</v>
+      </c>
+      <c r="E808" t="s">
+        <v>249</v>
+      </c>
+      <c r="F808">
+        <v>7</v>
+      </c>
+      <c r="G808">
+        <v>3.85</v>
+      </c>
+      <c r="H808">
+        <v>2276</v>
+      </c>
+    </row>
+    <row r="809" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A809" t="s">
+        <v>8</v>
+      </c>
+      <c r="B809" t="s">
+        <v>9</v>
+      </c>
+      <c r="C809" t="s">
+        <v>26</v>
+      </c>
+      <c r="D809" t="s">
+        <v>372</v>
+      </c>
+      <c r="E809" t="s">
+        <v>12</v>
+      </c>
+      <c r="F809">
+        <v>1</v>
+      </c>
+      <c r="G809">
+        <v>4.99</v>
+      </c>
+      <c r="H809">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="810" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A810" t="s">
+        <v>8</v>
+      </c>
+      <c r="B810" t="s">
+        <v>9</v>
+      </c>
+      <c r="C810" t="s">
+        <v>26</v>
+      </c>
+      <c r="D810" t="s">
+        <v>47</v>
+      </c>
+      <c r="E810" t="s">
+        <v>146</v>
+      </c>
+      <c r="F810">
+        <v>7</v>
+      </c>
+      <c r="G810">
+        <v>7</v>
+      </c>
+      <c r="H810">
+        <v>4997</v>
+      </c>
+    </row>
+    <row r="811" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A811" t="s">
+        <v>17</v>
+      </c>
+      <c r="B811" t="s">
+        <v>18</v>
+      </c>
+      <c r="C811" t="s">
+        <v>26</v>
+      </c>
+      <c r="D811" t="s">
+        <v>226</v>
+      </c>
+      <c r="E811" t="s">
+        <v>227</v>
+      </c>
+      <c r="F811">
+        <v>4</v>
+      </c>
+      <c r="G811">
+        <v>3.49</v>
+      </c>
+      <c r="H811">
+        <v>3693</v>
+      </c>
+    </row>
+    <row r="812" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A812" t="s">
+        <v>29</v>
+      </c>
+      <c r="B812" t="s">
+        <v>30</v>
+      </c>
+      <c r="C812" t="s">
+        <v>19</v>
+      </c>
+      <c r="D812" t="s">
+        <v>189</v>
+      </c>
+      <c r="E812" t="s">
+        <v>280</v>
+      </c>
+      <c r="F812">
+        <v>2</v>
+      </c>
+      <c r="G812">
+        <v>4</v>
+      </c>
+      <c r="H812">
+        <v>3312</v>
+      </c>
+    </row>
+    <row r="813" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A813" t="s">
+        <v>17</v>
+      </c>
+      <c r="B813" t="s">
+        <v>18</v>
+      </c>
+      <c r="C813" t="s">
+        <v>31</v>
+      </c>
+      <c r="D813" t="s">
+        <v>58</v>
+      </c>
+      <c r="E813" t="s">
+        <v>58</v>
+      </c>
+      <c r="F813">
+        <v>-3</v>
+      </c>
+      <c r="G813">
+        <v>5.05</v>
+      </c>
+      <c r="H813">
+        <v>1649</v>
+      </c>
+    </row>
+    <row r="814" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A814" t="s">
+        <v>17</v>
+      </c>
+      <c r="B814" t="s">
+        <v>18</v>
+      </c>
+      <c r="C814" t="s">
+        <v>19</v>
+      </c>
+      <c r="D814" t="s">
+        <v>350</v>
+      </c>
+      <c r="E814" t="s">
+        <v>204</v>
+      </c>
+      <c r="F814">
+        <v>-1</v>
+      </c>
+      <c r="G814">
+        <v>3.28</v>
+      </c>
+      <c r="H814">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="815" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A815" t="s">
+        <v>13</v>
+      </c>
+      <c r="B815" t="s">
+        <v>14</v>
+      </c>
+      <c r="C815" t="s">
+        <v>26</v>
+      </c>
+      <c r="D815" t="s">
+        <v>130</v>
+      </c>
+      <c r="E815" t="s">
+        <v>232</v>
+      </c>
+      <c r="F815">
+        <v>4</v>
+      </c>
+      <c r="G815">
+        <v>3.34</v>
+      </c>
+      <c r="H815">
+        <v>3921</v>
+      </c>
+    </row>
+    <row r="816" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A816" t="s">
+        <v>17</v>
+      </c>
+      <c r="B816" t="s">
+        <v>18</v>
+      </c>
+      <c r="C816" t="s">
+        <v>19</v>
+      </c>
+      <c r="D816" t="s">
+        <v>211</v>
+      </c>
+      <c r="E816" t="s">
+        <v>24</v>
+      </c>
+      <c r="F816">
+        <v>2</v>
+      </c>
+      <c r="G816">
+        <v>4.1100000000000003</v>
+      </c>
+      <c r="H816">
+        <v>2147</v>
+      </c>
+    </row>
+    <row r="817" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A817" t="s">
+        <v>8</v>
+      </c>
+      <c r="C817" t="s">
+        <v>31</v>
+      </c>
+      <c r="D817" t="s">
+        <v>162</v>
+      </c>
+      <c r="E817" t="s">
+        <v>162</v>
+      </c>
+      <c r="F817">
+        <v>2</v>
+      </c>
+      <c r="G817">
+        <v>3.76</v>
+      </c>
+      <c r="H817">
+        <v>4035</v>
+      </c>
+    </row>
+    <row r="818" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A818" t="s">
+        <v>8</v>
+      </c>
+      <c r="B818" t="s">
+        <v>9</v>
+      </c>
+      <c r="C818" t="s">
+        <v>26</v>
+      </c>
+      <c r="D818" t="s">
+        <v>104</v>
+      </c>
+      <c r="E818" t="s">
+        <v>43</v>
+      </c>
+      <c r="F818">
+        <v>2</v>
+      </c>
+      <c r="G818">
+        <v>3.76</v>
+      </c>
+      <c r="H818">
+        <v>4941</v>
+      </c>
+    </row>
+    <row r="819" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A819" t="s">
+        <v>29</v>
+      </c>
+      <c r="B819" t="s">
+        <v>30</v>
+      </c>
+      <c r="C819" t="s">
+        <v>31</v>
+      </c>
+      <c r="D819" t="s">
+        <v>176</v>
+      </c>
+      <c r="E819" t="s">
+        <v>140</v>
+      </c>
+      <c r="F819">
+        <v>0</v>
+      </c>
+      <c r="G819">
+        <v>3.74</v>
+      </c>
+      <c r="H819">
+        <v>1045</v>
+      </c>
+    </row>
+    <row r="820" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A820" t="s">
+        <v>8</v>
+      </c>
+      <c r="B820" t="s">
+        <v>9</v>
+      </c>
+      <c r="C820" t="s">
+        <v>26</v>
+      </c>
+      <c r="D820" t="s">
+        <v>240</v>
+      </c>
+      <c r="E820" t="s">
+        <v>377</v>
+      </c>
+      <c r="F820">
+        <v>2</v>
+      </c>
+      <c r="G820">
+        <v>4.1500000000000004</v>
+      </c>
+      <c r="H820">
+        <v>2199</v>
+      </c>
+    </row>
+    <row r="821" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A821" t="s">
+        <v>17</v>
+      </c>
+      <c r="B821" t="s">
+        <v>18</v>
+      </c>
+      <c r="C821" t="s">
+        <v>26</v>
+      </c>
+      <c r="D821" t="s">
+        <v>97</v>
+      </c>
+      <c r="E821" t="s">
+        <v>131</v>
+      </c>
+      <c r="F821">
+        <v>6</v>
+      </c>
+      <c r="G821">
+        <v>3</v>
+      </c>
+      <c r="H821">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="822" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A822" t="s">
+        <v>8</v>
+      </c>
+      <c r="B822" t="s">
+        <v>9</v>
+      </c>
+      <c r="C822" t="s">
+        <v>10</v>
+      </c>
+      <c r="D822" t="s">
+        <v>234</v>
+      </c>
+      <c r="E822" t="s">
+        <v>183</v>
+      </c>
+      <c r="F822">
+        <v>-5</v>
+      </c>
+      <c r="G822">
+        <v>3.71</v>
+      </c>
+      <c r="H822">
+        <v>4452</v>
+      </c>
+    </row>
+    <row r="823" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A823" t="s">
+        <v>8</v>
+      </c>
+      <c r="B823" t="s">
+        <v>9</v>
+      </c>
+      <c r="C823" t="s">
+        <v>36</v>
+      </c>
+      <c r="D823" t="s">
+        <v>272</v>
+      </c>
+      <c r="E823" t="s">
+        <v>203</v>
+      </c>
+      <c r="F823">
+        <v>1</v>
+      </c>
+      <c r="G823">
+        <v>4.21</v>
+      </c>
+      <c r="H823">
+        <v>3830</v>
+      </c>
+    </row>
+    <row r="824" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A824" t="s">
+        <v>17</v>
+      </c>
+      <c r="B824" t="s">
+        <v>18</v>
+      </c>
+      <c r="C824" t="s">
+        <v>15</v>
+      </c>
+      <c r="D824" t="s">
+        <v>211</v>
+      </c>
+      <c r="E824" t="s">
+        <v>190</v>
+      </c>
+      <c r="F824">
+        <v>-2</v>
+      </c>
+      <c r="G824">
+        <v>4.83</v>
+      </c>
+      <c r="H824">
+        <v>3594</v>
+      </c>
+    </row>
+    <row r="825" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A825" t="s">
+        <v>8</v>
+      </c>
+      <c r="B825" t="s">
+        <v>9</v>
+      </c>
+      <c r="C825" t="s">
+        <v>26</v>
+      </c>
+      <c r="D825" t="s">
+        <v>366</v>
+      </c>
+      <c r="E825" t="s">
+        <v>184</v>
+      </c>
+      <c r="F825">
+        <v>-1</v>
+      </c>
+      <c r="G825">
+        <v>3</v>
+      </c>
+      <c r="H825">
+        <v>1131</v>
+      </c>
+    </row>
+    <row r="826" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A826" t="s">
+        <v>8</v>
+      </c>
+      <c r="B826" t="s">
+        <v>9</v>
+      </c>
+      <c r="C826" t="s">
+        <v>26</v>
+      </c>
+      <c r="D826" t="s">
+        <v>299</v>
+      </c>
+      <c r="E826" t="s">
+        <v>193</v>
+      </c>
+      <c r="F826">
+        <v>7</v>
+      </c>
+      <c r="G826">
+        <v>4.6500000000000004</v>
+      </c>
+      <c r="H826">
+        <v>3139</v>
+      </c>
+    </row>
+    <row r="827" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B827" t="s">
+        <v>18</v>
+      </c>
+      <c r="C827" t="s">
+        <v>19</v>
+      </c>
+      <c r="E827" t="s">
+        <v>24</v>
+      </c>
+      <c r="F827">
+        <v>5</v>
+      </c>
+      <c r="H827">
+        <v>2151</v>
+      </c>
+    </row>
+    <row r="828" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A828" t="s">
+        <v>13</v>
+      </c>
+      <c r="B828" t="s">
+        <v>14</v>
+      </c>
+      <c r="C828" t="s">
+        <v>15</v>
+      </c>
+      <c r="D828" t="s">
+        <v>79</v>
+      </c>
+      <c r="E828" t="s">
+        <v>80</v>
+      </c>
+      <c r="F828">
+        <v>6</v>
+      </c>
+      <c r="G828">
+        <v>3.89</v>
+      </c>
+      <c r="H828">
+        <v>4445</v>
+      </c>
+    </row>
+    <row r="829" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A829" t="s">
+        <v>17</v>
+      </c>
+      <c r="B829" t="s">
+        <v>18</v>
+      </c>
+      <c r="C829" t="s">
+        <v>19</v>
+      </c>
+      <c r="D829" t="s">
+        <v>112</v>
+      </c>
+      <c r="E829" t="s">
+        <v>112</v>
+      </c>
+      <c r="F829">
+        <v>-1</v>
+      </c>
+      <c r="G829">
+        <v>4.2699999999999996</v>
+      </c>
+      <c r="H829">
+        <v>3918</v>
+      </c>
+    </row>
+    <row r="830" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A830" t="s">
+        <v>8</v>
+      </c>
+      <c r="B830" t="s">
+        <v>9</v>
+      </c>
+      <c r="C830" t="s">
+        <v>10</v>
+      </c>
+      <c r="D830" t="s">
+        <v>361</v>
+      </c>
+      <c r="E830" t="s">
+        <v>361</v>
+      </c>
+      <c r="F830">
+        <v>-1</v>
+      </c>
+      <c r="G830">
+        <v>5.24</v>
+      </c>
+      <c r="H830">
+        <v>2214</v>
+      </c>
+    </row>
+    <row r="831" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A831" t="s">
+        <v>17</v>
+      </c>
+      <c r="B831" t="s">
+        <v>18</v>
+      </c>
+      <c r="C831" t="s">
+        <v>36</v>
+      </c>
+      <c r="D831" t="s">
+        <v>158</v>
+      </c>
+      <c r="E831" t="s">
+        <v>159</v>
+      </c>
+      <c r="F831">
+        <v>1</v>
+      </c>
+      <c r="G831">
+        <v>3.3</v>
+      </c>
+      <c r="H831">
+        <v>3264</v>
+      </c>
+    </row>
+    <row r="832" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A832" t="s">
+        <v>29</v>
+      </c>
+      <c r="C832" t="s">
+        <v>10</v>
+      </c>
+      <c r="D832" t="s">
+        <v>333</v>
+      </c>
+      <c r="E832" t="s">
+        <v>74</v>
+      </c>
+      <c r="F832">
+        <v>6</v>
+      </c>
+      <c r="G832">
+        <v>4.55</v>
+      </c>
+      <c r="H832">
+        <v>1949</v>
+      </c>
+    </row>
+    <row r="833" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A833" t="s">
+        <v>8</v>
+      </c>
+      <c r="B833" t="s">
+        <v>9</v>
+      </c>
+      <c r="C833" t="s">
+        <v>19</v>
+      </c>
+      <c r="D833" t="s">
+        <v>80</v>
+      </c>
+      <c r="E833" t="s">
+        <v>348</v>
+      </c>
+      <c r="F833">
+        <v>3</v>
+      </c>
+      <c r="G833">
+        <v>3.63</v>
+      </c>
+      <c r="H833">
+        <v>4365</v>
+      </c>
+    </row>
+    <row r="834" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A834" t="s">
+        <v>17</v>
+      </c>
+      <c r="B834" t="s">
+        <v>18</v>
+      </c>
+      <c r="C834" t="s">
+        <v>26</v>
+      </c>
+      <c r="D834" t="s">
+        <v>193</v>
+      </c>
+      <c r="E834" t="s">
+        <v>158</v>
+      </c>
+      <c r="F834">
+        <v>4</v>
+      </c>
+      <c r="G834">
+        <v>3.64</v>
+      </c>
+      <c r="H834">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="835" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A835" t="s">
+        <v>17</v>
+      </c>
+      <c r="B835" t="s">
+        <v>18</v>
+      </c>
+      <c r="C835" t="s">
+        <v>36</v>
+      </c>
+      <c r="D835" t="s">
+        <v>87</v>
+      </c>
+      <c r="E835" t="s">
+        <v>155</v>
+      </c>
+      <c r="F835">
+        <v>6</v>
+      </c>
+      <c r="G835">
+        <v>3.42</v>
+      </c>
+      <c r="H835">
+        <v>4691</v>
+      </c>
+    </row>
+    <row r="836" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A836" t="s">
+        <v>17</v>
+      </c>
+      <c r="B836" t="s">
+        <v>18</v>
+      </c>
+      <c r="C836" t="s">
+        <v>15</v>
+      </c>
+      <c r="D836" t="s">
+        <v>178</v>
+      </c>
+      <c r="E836" t="s">
+        <v>322</v>
+      </c>
+      <c r="F836">
+        <v>-2</v>
+      </c>
+      <c r="G836">
+        <v>3.67</v>
+      </c>
+      <c r="H836">
+        <v>1385</v>
+      </c>
+    </row>
+    <row r="837" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A837" t="s">
+        <v>13</v>
+      </c>
+      <c r="B837" t="s">
+        <v>14</v>
+      </c>
+      <c r="C837" t="s">
+        <v>19</v>
+      </c>
+      <c r="D837" t="s">
+        <v>175</v>
+      </c>
+      <c r="E837" t="s">
+        <v>358</v>
+      </c>
+      <c r="F837">
+        <v>7</v>
+      </c>
+      <c r="G837">
+        <v>4.8099999999999996</v>
+      </c>
+      <c r="H837">
+        <v>3220</v>
+      </c>
+    </row>
+    <row r="838" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A838" t="s">
+        <v>8</v>
+      </c>
+      <c r="B838" t="s">
+        <v>9</v>
+      </c>
+      <c r="C838" t="s">
+        <v>26</v>
+      </c>
+      <c r="D838" t="s">
+        <v>299</v>
+      </c>
+      <c r="E838" t="s">
+        <v>193</v>
+      </c>
+      <c r="F838">
+        <v>3</v>
+      </c>
+      <c r="G838">
+        <v>4.25</v>
+      </c>
+      <c r="H838">
+        <v>3137</v>
+      </c>
+    </row>
+    <row r="839" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A839" t="s">
+        <v>29</v>
+      </c>
+      <c r="B839" t="s">
+        <v>30</v>
+      </c>
+      <c r="C839" t="s">
+        <v>10</v>
+      </c>
+      <c r="D839" t="s">
+        <v>179</v>
+      </c>
+      <c r="E839" t="s">
+        <v>179</v>
+      </c>
+      <c r="F839">
+        <v>2</v>
+      </c>
+      <c r="G839">
+        <v>4.03</v>
+      </c>
+      <c r="H839">
+        <v>2735</v>
+      </c>
+    </row>
+    <row r="840" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A840" t="s">
+        <v>17</v>
+      </c>
+      <c r="B840" t="s">
+        <v>18</v>
+      </c>
+      <c r="C840" t="s">
+        <v>15</v>
+      </c>
+      <c r="D840" t="s">
+        <v>87</v>
+      </c>
+      <c r="E840" t="s">
+        <v>147</v>
+      </c>
+      <c r="F840">
+        <v>5</v>
+      </c>
+      <c r="G840">
+        <v>4.18</v>
+      </c>
+      <c r="H840">
+        <v>3822</v>
+      </c>
+    </row>
+    <row r="841" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A841" t="s">
+        <v>13</v>
+      </c>
+      <c r="B841" t="s">
+        <v>14</v>
+      </c>
+      <c r="C841" t="s">
+        <v>36</v>
+      </c>
+      <c r="D841" t="s">
+        <v>208</v>
+      </c>
+      <c r="E841" t="s">
+        <v>208</v>
+      </c>
+      <c r="F841">
+        <v>0</v>
+      </c>
+      <c r="G841">
+        <v>4.88</v>
+      </c>
+      <c r="H841">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="842" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A842" t="s">
+        <v>29</v>
+      </c>
+      <c r="B842" t="s">
+        <v>30</v>
+      </c>
+      <c r="C842" t="s">
+        <v>19</v>
+      </c>
+      <c r="D842" t="s">
+        <v>378</v>
+      </c>
+      <c r="E842" t="s">
+        <v>344</v>
+      </c>
+      <c r="F842">
+        <v>-6</v>
+      </c>
+      <c r="G842">
+        <v>4.76</v>
+      </c>
+      <c r="H842">
+        <v>1303</v>
+      </c>
+    </row>
+    <row r="843" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A843" t="s">
+        <v>8</v>
+      </c>
+      <c r="B843" t="s">
+        <v>9</v>
+      </c>
+      <c r="C843" t="s">
+        <v>26</v>
+      </c>
+      <c r="D843" t="s">
+        <v>78</v>
+      </c>
+      <c r="E843" t="s">
+        <v>161</v>
+      </c>
+      <c r="F843">
+        <v>4</v>
+      </c>
+      <c r="G843">
+        <v>3.05</v>
+      </c>
+      <c r="H843">
+        <v>1688</v>
+      </c>
+    </row>
+    <row r="844" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A844" t="s">
+        <v>17</v>
+      </c>
+      <c r="B844" t="s">
+        <v>18</v>
+      </c>
+      <c r="C844" t="s">
+        <v>19</v>
+      </c>
+      <c r="D844" t="s">
+        <v>229</v>
+      </c>
+      <c r="E844" t="s">
+        <v>341</v>
+      </c>
+      <c r="F844">
+        <v>0</v>
+      </c>
+      <c r="G844">
+        <v>4.71</v>
+      </c>
+      <c r="H844">
+        <v>1131</v>
+      </c>
+    </row>
+    <row r="845" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A845" t="s">
+        <v>8</v>
+      </c>
+      <c r="B845" t="s">
+        <v>9</v>
+      </c>
+      <c r="C845" t="s">
+        <v>19</v>
+      </c>
+      <c r="D845" t="s">
+        <v>173</v>
+      </c>
+      <c r="E845" t="s">
+        <v>24</v>
+      </c>
+      <c r="F845">
+        <v>7</v>
+      </c>
+      <c r="G845">
+        <v>4.41</v>
+      </c>
+      <c r="H845">
+        <v>2432</v>
+      </c>
+    </row>
+    <row r="846" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A846" t="s">
+        <v>8</v>
+      </c>
+      <c r="B846" t="s">
+        <v>9</v>
+      </c>
+      <c r="C846" t="s">
+        <v>26</v>
+      </c>
+      <c r="D846" t="s">
+        <v>127</v>
+      </c>
+      <c r="E846" t="s">
+        <v>166</v>
+      </c>
+      <c r="F846">
+        <v>1</v>
+      </c>
+      <c r="G846">
+        <v>4.99</v>
+      </c>
+      <c r="H846">
+        <v>3567</v>
+      </c>
+    </row>
+    <row r="847" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A847" t="s">
+        <v>13</v>
+      </c>
+      <c r="C847" t="s">
+        <v>26</v>
+      </c>
+      <c r="D847" t="s">
+        <v>160</v>
+      </c>
+      <c r="E847" t="s">
+        <v>160</v>
+      </c>
+      <c r="F847">
+        <v>-4</v>
+      </c>
+      <c r="G847">
+        <v>4.83</v>
+      </c>
+      <c r="H847">
+        <v>1025</v>
+      </c>
+    </row>
+    <row r="848" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A848" t="s">
+        <v>8</v>
+      </c>
+      <c r="B848" t="s">
+        <v>9</v>
+      </c>
+      <c r="C848" t="s">
+        <v>19</v>
+      </c>
+      <c r="D848" t="s">
+        <v>188</v>
+      </c>
+      <c r="E848" t="s">
+        <v>319</v>
+      </c>
+      <c r="F848">
+        <v>7</v>
+      </c>
+      <c r="G848">
+        <v>4.1900000000000004</v>
+      </c>
+      <c r="H848">
+        <v>2583</v>
+      </c>
+    </row>
+    <row r="849" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A849" t="s">
+        <v>8</v>
+      </c>
+      <c r="B849" t="s">
+        <v>9</v>
+      </c>
+      <c r="C849" t="s">
+        <v>19</v>
+      </c>
+      <c r="D849" t="s">
+        <v>348</v>
+      </c>
+      <c r="E849" t="s">
+        <v>368</v>
+      </c>
+      <c r="F849">
+        <v>5</v>
+      </c>
+      <c r="G849">
+        <v>4.2300000000000004</v>
+      </c>
+      <c r="H849">
+        <v>4471</v>
+      </c>
+    </row>
+    <row r="850" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A850" t="s">
+        <v>13</v>
+      </c>
+      <c r="B850" t="s">
+        <v>14</v>
+      </c>
+      <c r="C850" t="s">
+        <v>15</v>
+      </c>
+      <c r="D850" t="s">
+        <v>56</v>
+      </c>
+      <c r="E850" t="s">
+        <v>262</v>
+      </c>
+      <c r="F850">
+        <v>7</v>
+      </c>
+      <c r="G850">
+        <v>4.22</v>
+      </c>
+      <c r="H850">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="851" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A851" t="s">
+        <v>17</v>
+      </c>
+      <c r="B851" t="s">
+        <v>18</v>
+      </c>
+      <c r="C851" t="s">
+        <v>19</v>
+      </c>
+      <c r="D851" t="s">
+        <v>208</v>
+      </c>
+      <c r="E851" t="s">
+        <v>380</v>
+      </c>
+      <c r="F851">
+        <v>10</v>
+      </c>
+      <c r="G851">
+        <v>7</v>
+      </c>
+      <c r="H851">
+        <v>3163</v>
+      </c>
+    </row>
+    <row r="852" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B852" t="s">
+        <v>14</v>
+      </c>
+      <c r="C852" t="s">
+        <v>36</v>
+      </c>
+      <c r="E852" t="s">
+        <v>24</v>
+      </c>
+      <c r="F852">
+        <v>1</v>
+      </c>
+      <c r="H852">
+        <v>2459</v>
+      </c>
+    </row>
+    <row r="853" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A853" t="s">
+        <v>29</v>
+      </c>
+      <c r="B853" t="s">
+        <v>30</v>
+      </c>
+      <c r="C853" t="s">
+        <v>19</v>
+      </c>
+      <c r="D853" t="s">
+        <v>56</v>
+      </c>
+      <c r="E853" t="s">
+        <v>56</v>
+      </c>
+      <c r="F853">
+        <v>1</v>
+      </c>
+      <c r="G853">
+        <v>4.4400000000000004</v>
+      </c>
+      <c r="H853">
+        <v>1328</v>
+      </c>
+    </row>
+    <row r="854" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A854" t="s">
+        <v>13</v>
+      </c>
+      <c r="B854" t="s">
+        <v>14</v>
+      </c>
+      <c r="C854" t="s">
+        <v>15</v>
+      </c>
+      <c r="D854" t="s">
+        <v>126</v>
+      </c>
+      <c r="E854" t="s">
+        <v>77</v>
+      </c>
+      <c r="F854">
+        <v>5</v>
+      </c>
+      <c r="G854">
+        <v>3</v>
+      </c>
+      <c r="H854">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="855" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A855" t="s">
+        <v>29</v>
+      </c>
+      <c r="B855" t="s">
+        <v>30</v>
+      </c>
+      <c r="C855" t="s">
+        <v>31</v>
+      </c>
+      <c r="D855" t="s">
+        <v>90</v>
+      </c>
+      <c r="E855" t="s">
+        <v>234</v>
+      </c>
+      <c r="F855">
+        <v>-2</v>
+      </c>
+      <c r="G855">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="H855">
+        <v>3877</v>
+      </c>
+    </row>
+    <row r="856" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A856" t="s">
+        <v>13</v>
+      </c>
+      <c r="B856" t="s">
+        <v>14</v>
+      </c>
+      <c r="C856" t="s">
+        <v>15</v>
+      </c>
+      <c r="D856" t="s">
+        <v>56</v>
+      </c>
+      <c r="E856" t="s">
+        <v>262</v>
+      </c>
+      <c r="F856">
+        <v>10</v>
+      </c>
+      <c r="G856">
+        <v>4.32</v>
+      </c>
+      <c r="H856">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="857" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A857" t="s">
+        <v>17</v>
+      </c>
+      <c r="B857" t="s">
+        <v>18</v>
+      </c>
+      <c r="C857" t="s">
+        <v>31</v>
+      </c>
+      <c r="D857" t="s">
+        <v>280</v>
+      </c>
+      <c r="E857" t="s">
+        <v>283</v>
+      </c>
+      <c r="F857">
+        <v>7</v>
+      </c>
+      <c r="G857">
+        <v>3.31</v>
+      </c>
+      <c r="H857">
+        <v>4167</v>
+      </c>
+    </row>
+    <row r="858" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A858" t="s">
+        <v>29</v>
+      </c>
+      <c r="B858" t="s">
+        <v>30</v>
+      </c>
+      <c r="C858" t="s">
+        <v>10</v>
+      </c>
+      <c r="D858" t="s">
+        <v>295</v>
+      </c>
+      <c r="E858" t="s">
+        <v>254</v>
+      </c>
+      <c r="F858">
+        <v>1</v>
+      </c>
+      <c r="G858">
+        <v>3.32</v>
+      </c>
+      <c r="H858">
+        <v>1612</v>
+      </c>
+    </row>
+    <row r="859" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A859" t="s">
+        <v>17</v>
+      </c>
+      <c r="B859" t="s">
+        <v>18</v>
+      </c>
+      <c r="C859" t="s">
+        <v>36</v>
+      </c>
+      <c r="D859" t="s">
+        <v>121</v>
+      </c>
+      <c r="E859" t="s">
+        <v>121</v>
+      </c>
+      <c r="F859">
+        <v>-1</v>
+      </c>
+      <c r="G859">
+        <v>3.21</v>
+      </c>
+      <c r="H859">
+        <v>1839</v>
+      </c>
+    </row>
+    <row r="860" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A860" t="s">
+        <v>29</v>
+      </c>
+      <c r="B860" t="s">
+        <v>30</v>
+      </c>
+      <c r="C860" t="s">
+        <v>19</v>
+      </c>
+      <c r="D860" t="s">
+        <v>226</v>
+      </c>
+      <c r="E860" t="s">
+        <v>268</v>
+      </c>
+      <c r="F860">
+        <v>2</v>
+      </c>
+      <c r="G860">
+        <v>3.35</v>
+      </c>
+      <c r="H860">
+        <v>4846</v>
+      </c>
+    </row>
+    <row r="861" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A861" t="s">
+        <v>13</v>
+      </c>
+      <c r="B861" t="s">
+        <v>14</v>
+      </c>
+      <c r="C861" t="s">
+        <v>19</v>
+      </c>
+      <c r="D861" t="s">
+        <v>231</v>
+      </c>
+      <c r="E861" t="s">
+        <v>42</v>
+      </c>
+      <c r="F861">
+        <v>0</v>
+      </c>
+      <c r="G861">
+        <v>3.33</v>
+      </c>
+      <c r="H861">
+        <v>2940</v>
+      </c>
+    </row>
+    <row r="862" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A862" t="s">
+        <v>29</v>
+      </c>
+      <c r="C862" t="s">
+        <v>26</v>
+      </c>
+      <c r="D862" t="s">
+        <v>317</v>
+      </c>
+      <c r="E862" t="s">
+        <v>100</v>
+      </c>
+      <c r="F862">
+        <v>-4</v>
+      </c>
+      <c r="G862">
+        <v>3.91</v>
+      </c>
+      <c r="H862">
+        <v>3451</v>
+      </c>
+    </row>
+    <row r="863" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A863" t="s">
+        <v>13</v>
+      </c>
+      <c r="B863" t="s">
+        <v>14</v>
+      </c>
+      <c r="C863" t="s">
+        <v>15</v>
+      </c>
+      <c r="D863" t="s">
+        <v>43</v>
+      </c>
+      <c r="E863" t="s">
+        <v>44</v>
+      </c>
+      <c r="F863">
+        <v>0</v>
+      </c>
+      <c r="G863">
+        <v>4.79</v>
+      </c>
+      <c r="H863">
+        <v>3234</v>
+      </c>
+    </row>
+    <row r="864" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A864" t="s">
+        <v>17</v>
+      </c>
+      <c r="B864" t="s">
+        <v>18</v>
+      </c>
+      <c r="C864" t="s">
+        <v>26</v>
+      </c>
+      <c r="D864" t="s">
+        <v>61</v>
+      </c>
+      <c r="E864" t="s">
+        <v>43</v>
+      </c>
+      <c r="F864">
+        <v>4</v>
+      </c>
+      <c r="G864">
+        <v>3.13</v>
+      </c>
+      <c r="H864">
+        <v>2853</v>
+      </c>
+    </row>
+    <row r="865" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A865" t="s">
+        <v>8</v>
+      </c>
+      <c r="B865" t="s">
+        <v>9</v>
+      </c>
+      <c r="C865" t="s">
+        <v>15</v>
+      </c>
+      <c r="D865" t="s">
+        <v>166</v>
+      </c>
+      <c r="E865" t="s">
+        <v>233</v>
+      </c>
+      <c r="F865">
+        <v>3</v>
+      </c>
+      <c r="G865">
+        <v>3.9</v>
+      </c>
+      <c r="H865">
+        <v>3629</v>
+      </c>
+    </row>
+    <row r="866" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A866" t="s">
+        <v>17</v>
+      </c>
+      <c r="B866" t="s">
+        <v>18</v>
+      </c>
+      <c r="C866" t="s">
+        <v>15</v>
+      </c>
+      <c r="D866" t="s">
+        <v>211</v>
+      </c>
+      <c r="E866" t="s">
+        <v>190</v>
+      </c>
+      <c r="F866">
+        <v>-1</v>
+      </c>
+      <c r="G866">
+        <v>5.16</v>
+      </c>
+      <c r="H866">
+        <v>3594</v>
+      </c>
+    </row>
+    <row r="867" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A867" t="s">
+        <v>17</v>
+      </c>
+      <c r="B867" t="s">
+        <v>18</v>
+      </c>
+      <c r="C867" t="s">
+        <v>36</v>
+      </c>
+      <c r="D867" t="s">
+        <v>144</v>
+      </c>
+      <c r="E867" t="s">
+        <v>211</v>
+      </c>
+      <c r="F867">
+        <v>6</v>
+      </c>
+      <c r="G867">
+        <v>3</v>
+      </c>
+      <c r="H867">
+        <v>4890</v>
+      </c>
+    </row>
+    <row r="868" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A868" t="s">
+        <v>17</v>
+      </c>
+      <c r="B868" t="s">
+        <v>18</v>
+      </c>
+      <c r="C868" t="s">
+        <v>19</v>
+      </c>
+      <c r="D868" t="s">
+        <v>123</v>
+      </c>
+      <c r="E868" t="s">
+        <v>303</v>
+      </c>
+      <c r="F868">
+        <v>9</v>
+      </c>
+      <c r="G868">
+        <v>4.12</v>
+      </c>
+      <c r="H868">
+        <v>1565</v>
+      </c>
+    </row>
+    <row r="869" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A869" t="s">
+        <v>29</v>
+      </c>
+      <c r="B869" t="s">
+        <v>30</v>
+      </c>
+      <c r="C869" t="s">
+        <v>19</v>
+      </c>
+      <c r="D869" t="s">
+        <v>114</v>
+      </c>
+      <c r="E869" t="s">
+        <v>235</v>
+      </c>
+      <c r="F869">
+        <v>4</v>
+      </c>
+      <c r="G869">
+        <v>4.29</v>
+      </c>
+      <c r="H869">
+        <v>4548</v>
+      </c>
+    </row>
+    <row r="870" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A870" t="s">
+        <v>13</v>
+      </c>
+      <c r="B870" t="s">
+        <v>14</v>
+      </c>
+      <c r="C870" t="s">
+        <v>10</v>
+      </c>
+      <c r="D870" t="s">
+        <v>154</v>
+      </c>
+      <c r="E870" t="s">
+        <v>155</v>
+      </c>
+      <c r="F870">
+        <v>8</v>
+      </c>
+      <c r="G870">
+        <v>5</v>
+      </c>
+      <c r="H870">
+        <v>2938</v>
+      </c>
+    </row>
+    <row r="871" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A871" t="s">
+        <v>17</v>
+      </c>
+      <c r="B871" t="s">
+        <v>18</v>
+      </c>
+      <c r="C871" t="s">
+        <v>19</v>
+      </c>
+      <c r="D871" t="s">
+        <v>20</v>
+      </c>
+      <c r="E871" t="s">
+        <v>20</v>
+      </c>
+      <c r="F871">
+        <v>-3</v>
+      </c>
+      <c r="G871">
+        <v>3.1</v>
+      </c>
+      <c r="H871">
+        <v>1528</v>
+      </c>
+    </row>
+    <row r="872" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A872" t="s">
+        <v>29</v>
+      </c>
+      <c r="B872" t="s">
+        <v>30</v>
+      </c>
+      <c r="C872" t="s">
+        <v>15</v>
+      </c>
+      <c r="D872" t="s">
+        <v>152</v>
+      </c>
+      <c r="E872" t="s">
+        <v>152</v>
+      </c>
+      <c r="F872">
+        <v>0</v>
+      </c>
+      <c r="G872">
+        <v>2.88</v>
+      </c>
+      <c r="H872">
+        <v>4478</v>
+      </c>
+    </row>
+    <row r="873" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A873" t="s">
+        <v>8</v>
+      </c>
+      <c r="B873" t="s">
+        <v>9</v>
+      </c>
+      <c r="C873" t="s">
+        <v>31</v>
+      </c>
+      <c r="D873" t="s">
+        <v>230</v>
+      </c>
+      <c r="E873" t="s">
+        <v>230</v>
+      </c>
+      <c r="F873">
+        <v>2</v>
+      </c>
+      <c r="G873">
+        <v>3.83</v>
+      </c>
+      <c r="H873">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="874" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A874" t="s">
+        <v>13</v>
+      </c>
+      <c r="B874" t="s">
+        <v>14</v>
+      </c>
+      <c r="C874" t="s">
+        <v>19</v>
+      </c>
+      <c r="D874" t="s">
+        <v>298</v>
+      </c>
+      <c r="E874" t="s">
+        <v>359</v>
+      </c>
+      <c r="F874">
+        <v>2</v>
+      </c>
+      <c r="G874">
+        <v>5.12</v>
+      </c>
+      <c r="H874">
+        <v>4420</v>
+      </c>
+    </row>
+    <row r="875" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A875" t="s">
+        <v>29</v>
+      </c>
+      <c r="B875" t="s">
+        <v>30</v>
+      </c>
+      <c r="C875" t="s">
+        <v>15</v>
+      </c>
+      <c r="D875" t="s">
+        <v>145</v>
+      </c>
+      <c r="E875" t="s">
+        <v>80</v>
+      </c>
+      <c r="F875">
+        <v>4</v>
+      </c>
+      <c r="G875">
+        <v>4.07</v>
+      </c>
+      <c r="H875">
+        <v>2407</v>
+      </c>
+    </row>
+    <row r="876" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A876" t="s">
+        <v>8</v>
+      </c>
+      <c r="B876" t="s">
+        <v>9</v>
+      </c>
+      <c r="C876" t="s">
+        <v>31</v>
+      </c>
+      <c r="D876" t="s">
+        <v>323</v>
+      </c>
+      <c r="E876" t="s">
+        <v>189</v>
+      </c>
+      <c r="F876">
+        <v>3</v>
+      </c>
+      <c r="G876">
+        <v>2.99</v>
+      </c>
+      <c r="H876">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="877" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="C877" t="s">
+        <v>15</v>
+      </c>
+      <c r="E877" t="s">
+        <v>93</v>
+      </c>
+      <c r="F877">
+        <v>3</v>
+      </c>
+      <c r="H877">
+        <v>2566</v>
+      </c>
+    </row>
+    <row r="878" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A878" t="s">
+        <v>13</v>
+      </c>
+      <c r="B878" t="s">
+        <v>14</v>
+      </c>
+      <c r="C878" t="s">
+        <v>31</v>
+      </c>
+      <c r="D878" t="s">
+        <v>237</v>
+      </c>
+      <c r="E878" t="s">
+        <v>237</v>
+      </c>
+      <c r="F878">
+        <v>-3</v>
+      </c>
+      <c r="G878">
+        <v>4.3099999999999996</v>
+      </c>
+      <c r="H878">
+        <v>4546</v>
+      </c>
+    </row>
+    <row r="879" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A879" t="s">
+        <v>29</v>
+      </c>
+      <c r="B879" t="s">
+        <v>30</v>
+      </c>
+      <c r="C879" t="s">
+        <v>31</v>
+      </c>
+      <c r="D879" t="s">
+        <v>151</v>
+      </c>
+      <c r="E879" t="s">
+        <v>235</v>
+      </c>
+      <c r="F879">
+        <v>4</v>
+      </c>
+      <c r="G879">
+        <v>3.78</v>
+      </c>
+      <c r="H879">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="880" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A880" t="s">
+        <v>17</v>
+      </c>
+      <c r="B880" t="s">
+        <v>18</v>
+      </c>
+      <c r="C880" t="s">
+        <v>10</v>
+      </c>
+      <c r="D880" t="s">
+        <v>282</v>
+      </c>
+      <c r="E880" t="s">
+        <v>282</v>
+      </c>
+      <c r="F880">
+        <v>-3</v>
+      </c>
+      <c r="G880">
+        <v>4.21</v>
+      </c>
+      <c r="H880">
+        <v>4564</v>
+      </c>
+    </row>
+    <row r="881" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A881" t="s">
+        <v>29</v>
+      </c>
+      <c r="B881" t="s">
+        <v>30</v>
+      </c>
+      <c r="C881" t="s">
+        <v>31</v>
+      </c>
+      <c r="D881" t="s">
+        <v>39</v>
+      </c>
+      <c r="E881" t="s">
+        <v>62</v>
+      </c>
+      <c r="F881">
+        <v>7</v>
+      </c>
+      <c r="G881">
+        <v>3.44</v>
+      </c>
+      <c r="H881">
+        <v>1634</v>
+      </c>
+    </row>
+    <row r="882" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A882" t="s">
+        <v>17</v>
+      </c>
+      <c r="B882" t="s">
+        <v>18</v>
+      </c>
+      <c r="C882" t="s">
+        <v>15</v>
+      </c>
+      <c r="D882" t="s">
+        <v>90</v>
+      </c>
+      <c r="E882" t="s">
+        <v>90</v>
+      </c>
+      <c r="F882">
+        <v>-3</v>
+      </c>
+      <c r="G882">
+        <v>5.0199999999999996</v>
+      </c>
+      <c r="H882">
+        <v>1542</v>
+      </c>
+    </row>
+    <row r="883" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A883" t="s">
+        <v>17</v>
+      </c>
+      <c r="B883" t="s">
+        <v>18</v>
+      </c>
+      <c r="C883" t="s">
+        <v>19</v>
+      </c>
+      <c r="D883" t="s">
+        <v>77</v>
+      </c>
+      <c r="E883" t="s">
+        <v>78</v>
+      </c>
+      <c r="F883">
+        <v>-1</v>
+      </c>
+      <c r="G883">
+        <v>4.7300000000000004</v>
+      </c>
+      <c r="H883">
+        <v>1796</v>
+      </c>
+    </row>
+    <row r="884" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A884" t="s">
+        <v>8</v>
+      </c>
+      <c r="B884" t="s">
+        <v>9</v>
+      </c>
+      <c r="C884" t="s">
+        <v>36</v>
+      </c>
+      <c r="D884" t="s">
+        <v>157</v>
+      </c>
+      <c r="E884" t="s">
+        <v>157</v>
+      </c>
+      <c r="F884">
+        <v>0</v>
+      </c>
+      <c r="G884">
+        <v>4.75</v>
+      </c>
+      <c r="H884">
+        <v>3695</v>
+      </c>
+    </row>
+    <row r="885" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A885" t="s">
+        <v>13</v>
+      </c>
+      <c r="B885" t="s">
+        <v>14</v>
+      </c>
+      <c r="C885" t="s">
+        <v>31</v>
+      </c>
+      <c r="D885" t="s">
+        <v>345</v>
+      </c>
+      <c r="E885" t="s">
+        <v>148</v>
+      </c>
+      <c r="F885">
+        <v>2</v>
+      </c>
+      <c r="G885">
+        <v>3.39</v>
+      </c>
+      <c r="H885">
+        <v>4743</v>
+      </c>
+    </row>
+    <row r="886" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A886" t="s">
+        <v>13</v>
+      </c>
+      <c r="B886" t="s">
+        <v>14</v>
+      </c>
+      <c r="C886" t="s">
+        <v>15</v>
+      </c>
+      <c r="D886" t="s">
+        <v>43</v>
+      </c>
+      <c r="E886" t="s">
+        <v>44</v>
+      </c>
+      <c r="F886">
+        <v>4</v>
+      </c>
+      <c r="G886">
+        <v>4.9800000000000004</v>
+      </c>
+      <c r="H886">
+        <v>3238</v>
+      </c>
+    </row>
+    <row r="887" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A887" t="s">
+        <v>13</v>
+      </c>
+      <c r="B887" t="s">
+        <v>14</v>
+      </c>
+      <c r="C887" t="s">
+        <v>26</v>
+      </c>
+      <c r="D887" t="s">
+        <v>146</v>
+      </c>
+      <c r="E887" t="s">
+        <v>204</v>
+      </c>
+      <c r="F887">
+        <v>2</v>
+      </c>
+      <c r="G887">
+        <v>5.01</v>
+      </c>
+      <c r="H887">
+        <v>3984</v>
+      </c>
+    </row>
+    <row r="888" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A888" t="s">
+        <v>17</v>
+      </c>
+      <c r="B888" t="s">
+        <v>18</v>
+      </c>
+      <c r="C888" t="s">
+        <v>26</v>
+      </c>
+      <c r="D888" t="s">
+        <v>116</v>
+      </c>
+      <c r="E888" t="s">
+        <v>298</v>
+      </c>
+      <c r="F888">
+        <v>-2</v>
+      </c>
+      <c r="G888">
+        <v>4.54</v>
+      </c>
+      <c r="H888">
+        <v>4798</v>
+      </c>
+    </row>
+    <row r="889" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A889" t="s">
+        <v>13</v>
+      </c>
+      <c r="B889" t="s">
+        <v>14</v>
+      </c>
+      <c r="C889" t="s">
+        <v>15</v>
+      </c>
+      <c r="D889" t="s">
+        <v>150</v>
+      </c>
+      <c r="E889" t="s">
+        <v>151</v>
+      </c>
+      <c r="F889">
+        <v>1</v>
+      </c>
+      <c r="G889">
+        <v>4.45</v>
+      </c>
+      <c r="H889">
+        <v>4271</v>
+      </c>
+    </row>
+    <row r="890" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A890" t="s">
+        <v>29</v>
+      </c>
+      <c r="B890" t="s">
+        <v>30</v>
+      </c>
+      <c r="C890" t="s">
+        <v>36</v>
+      </c>
+      <c r="D890" t="s">
+        <v>240</v>
+      </c>
+      <c r="E890" t="s">
+        <v>110</v>
+      </c>
+      <c r="F890">
+        <v>1</v>
+      </c>
+      <c r="G890">
+        <v>3.11</v>
+      </c>
+      <c r="H890">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="891" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A891" t="s">
+        <v>8</v>
+      </c>
+      <c r="B891" t="s">
+        <v>9</v>
+      </c>
+      <c r="C891" t="s">
+        <v>19</v>
+      </c>
+      <c r="D891" t="s">
+        <v>354</v>
+      </c>
+      <c r="E891" t="s">
+        <v>336</v>
+      </c>
+      <c r="F891">
+        <v>7</v>
+      </c>
+      <c r="G891">
+        <v>3.55</v>
+      </c>
+      <c r="H891">
+        <v>1630</v>
+      </c>
+    </row>
+    <row r="892" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A892" t="s">
+        <v>29</v>
+      </c>
+      <c r="C892" t="s">
+        <v>19</v>
+      </c>
+      <c r="D892" t="s">
+        <v>35</v>
+      </c>
+      <c r="E892" t="s">
+        <v>35</v>
+      </c>
+      <c r="F892">
+        <v>-1</v>
+      </c>
+      <c r="G892">
+        <v>3.41</v>
+      </c>
+      <c r="H892">
+        <v>976</v>
+      </c>
+    </row>
+    <row r="893" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A893" t="s">
+        <v>13</v>
+      </c>
+      <c r="B893" t="s">
+        <v>14</v>
+      </c>
+      <c r="C893" t="s">
+        <v>26</v>
+      </c>
+      <c r="D893" t="s">
+        <v>52</v>
+      </c>
+      <c r="E893" t="s">
+        <v>154</v>
+      </c>
+      <c r="F893">
+        <v>7</v>
+      </c>
+      <c r="G893">
+        <v>3.72</v>
+      </c>
+      <c r="H893">
+        <v>2822</v>
+      </c>
+    </row>
+    <row r="894" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A894" t="s">
+        <v>17</v>
+      </c>
+      <c r="B894" t="s">
+        <v>18</v>
+      </c>
+      <c r="C894" t="s">
+        <v>19</v>
+      </c>
+      <c r="D894" t="s">
+        <v>292</v>
+      </c>
+      <c r="E894" t="s">
+        <v>69</v>
+      </c>
+      <c r="F894">
+        <v>3</v>
+      </c>
+      <c r="G894">
+        <v>4.29</v>
+      </c>
+      <c r="H894">
+        <v>2937</v>
+      </c>
+    </row>
+    <row r="895" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A895" t="s">
+        <v>17</v>
+      </c>
+      <c r="B895" t="s">
+        <v>18</v>
+      </c>
+      <c r="C895" t="s">
+        <v>31</v>
+      </c>
+      <c r="D895" t="s">
+        <v>63</v>
+      </c>
+      <c r="E895" t="s">
+        <v>63</v>
+      </c>
+      <c r="F895">
+        <v>-4</v>
+      </c>
+      <c r="G895">
+        <v>3.48</v>
+      </c>
+      <c r="H895">
+        <v>1665</v>
+      </c>
+    </row>
+    <row r="896" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A896" t="s">
+        <v>13</v>
+      </c>
+      <c r="B896" t="s">
+        <v>14</v>
+      </c>
+      <c r="C896" t="s">
+        <v>31</v>
+      </c>
+      <c r="D896" t="s">
+        <v>230</v>
+      </c>
+      <c r="E896" t="s">
+        <v>202</v>
+      </c>
+      <c r="F896">
+        <v>7</v>
+      </c>
+      <c r="G896">
+        <v>3.97</v>
+      </c>
+      <c r="H896">
+        <v>1271</v>
+      </c>
+    </row>
+    <row r="897" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A897" t="s">
+        <v>13</v>
+      </c>
+      <c r="B897" t="s">
+        <v>14</v>
+      </c>
+      <c r="C897" t="s">
+        <v>15</v>
+      </c>
+      <c r="D897" t="s">
+        <v>205</v>
+      </c>
+      <c r="E897" t="s">
+        <v>289</v>
+      </c>
+      <c r="F897">
+        <v>9</v>
+      </c>
+      <c r="G897">
+        <v>3.41</v>
+      </c>
+      <c r="H897">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="898" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A898" t="s">
+        <v>17</v>
+      </c>
+      <c r="B898" t="s">
+        <v>18</v>
+      </c>
+      <c r="C898" t="s">
+        <v>36</v>
+      </c>
+      <c r="D898" t="s">
+        <v>86</v>
+      </c>
+      <c r="E898" t="s">
+        <v>86</v>
+      </c>
+      <c r="F898">
+        <v>-2</v>
+      </c>
+      <c r="G898">
+        <v>3.04</v>
+      </c>
+      <c r="H898">
+        <v>1972</v>
+      </c>
+    </row>
+    <row r="899" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A899" t="s">
+        <v>17</v>
+      </c>
+      <c r="B899" t="s">
+        <v>18</v>
+      </c>
+      <c r="C899" t="s">
+        <v>36</v>
+      </c>
+      <c r="D899" t="s">
+        <v>329</v>
+      </c>
+      <c r="E899" t="s">
+        <v>272</v>
+      </c>
+      <c r="F899">
+        <v>5</v>
+      </c>
+      <c r="G899">
+        <v>4.1399999999999997</v>
+      </c>
+      <c r="H899">
+        <v>3101</v>
+      </c>
+    </row>
+    <row r="900" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A900" t="s">
+        <v>8</v>
+      </c>
+      <c r="B900" t="s">
+        <v>9</v>
+      </c>
+      <c r="C900" t="s">
+        <v>26</v>
+      </c>
+      <c r="D900" t="s">
+        <v>240</v>
+      </c>
+      <c r="E900" t="s">
+        <v>377</v>
+      </c>
+      <c r="F900">
+        <v>1</v>
+      </c>
+      <c r="G900">
+        <v>3.75</v>
+      </c>
+      <c r="H900">
+        <v>2200</v>
+      </c>
+    </row>
+    <row r="901" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A901" t="s">
+        <v>17</v>
+      </c>
+      <c r="B901" t="s">
+        <v>18</v>
+      </c>
+      <c r="C901" t="s">
+        <v>19</v>
+      </c>
+      <c r="D901" t="s">
+        <v>171</v>
+      </c>
+      <c r="E901" t="s">
+        <v>284</v>
+      </c>
+      <c r="F901">
+        <v>-2</v>
+      </c>
+      <c r="G901">
+        <v>4.42</v>
+      </c>
+      <c r="H901">
+        <v>3826</v>
+      </c>
+    </row>
+    <row r="902" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B902" t="s">
+        <v>30</v>
+      </c>
+      <c r="C902" t="s">
+        <v>15</v>
+      </c>
+      <c r="E902" t="s">
+        <v>152</v>
+      </c>
+      <c r="F902">
+        <v>-3</v>
+      </c>
+      <c r="H902">
+        <v>4480</v>
+      </c>
+    </row>
+    <row r="903" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A903" t="s">
+        <v>29</v>
+      </c>
+      <c r="B903" t="s">
+        <v>30</v>
+      </c>
+      <c r="C903" t="s">
+        <v>31</v>
+      </c>
+      <c r="D903" t="s">
+        <v>315</v>
+      </c>
+      <c r="E903" t="s">
+        <v>305</v>
+      </c>
+      <c r="F903">
+        <v>7</v>
+      </c>
+      <c r="G903">
+        <v>2</v>
+      </c>
+      <c r="H903">
+        <v>1683</v>
+      </c>
+    </row>
+    <row r="904" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A904" t="s">
+        <v>29</v>
+      </c>
+      <c r="B904" t="s">
+        <v>30</v>
+      </c>
+      <c r="C904" t="s">
+        <v>15</v>
+      </c>
+      <c r="D904" t="s">
+        <v>187</v>
+      </c>
+      <c r="E904" t="s">
+        <v>228</v>
+      </c>
+      <c r="F904">
+        <v>0</v>
+      </c>
+      <c r="G904">
+        <v>3.4</v>
+      </c>
+      <c r="H904">
+        <v>4675</v>
+      </c>
+    </row>
+    <row r="905" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A905" t="s">
+        <v>13</v>
+      </c>
+      <c r="B905" t="s">
+        <v>14</v>
+      </c>
+      <c r="C905" t="s">
+        <v>31</v>
+      </c>
+      <c r="D905" t="s">
+        <v>336</v>
+      </c>
+      <c r="E905" t="s">
+        <v>71</v>
+      </c>
+      <c r="F905">
+        <v>4</v>
+      </c>
+      <c r="G905">
+        <v>2.88</v>
+      </c>
+      <c r="H905">
+        <v>1126</v>
+      </c>
+    </row>
+    <row r="906" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A906" t="s">
+        <v>17</v>
+      </c>
+      <c r="B906" t="s">
+        <v>18</v>
+      </c>
+      <c r="C906" t="s">
+        <v>26</v>
+      </c>
+      <c r="D906" t="s">
+        <v>50</v>
+      </c>
+      <c r="E906" t="s">
+        <v>101</v>
+      </c>
+      <c r="F906">
+        <v>5</v>
+      </c>
+      <c r="G906">
+        <v>2.97</v>
+      </c>
+      <c r="H906">
+        <v>1865</v>
+      </c>
+    </row>
+    <row r="907" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A907" t="s">
+        <v>29</v>
+      </c>
+      <c r="C907" t="s">
+        <v>15</v>
+      </c>
+      <c r="D907" t="s">
+        <v>136</v>
+      </c>
+      <c r="E907" t="s">
+        <v>149</v>
+      </c>
+      <c r="F907">
+        <v>8</v>
+      </c>
+      <c r="G907">
+        <v>8</v>
+      </c>
+      <c r="H907">
+        <v>3570</v>
+      </c>
+    </row>
+    <row r="908" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A908" t="s">
+        <v>29</v>
+      </c>
+      <c r="B908" t="s">
+        <v>30</v>
+      </c>
+      <c r="C908" t="s">
+        <v>26</v>
+      </c>
+      <c r="D908" t="s">
+        <v>236</v>
+      </c>
+      <c r="E908" t="s">
+        <v>237</v>
+      </c>
+      <c r="F908">
+        <v>4</v>
+      </c>
+      <c r="G908">
+        <v>4</v>
+      </c>
+      <c r="H908">
+        <v>4896</v>
+      </c>
+    </row>
+    <row r="909" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A909" t="s">
+        <v>29</v>
+      </c>
+      <c r="B909" t="s">
+        <v>30</v>
+      </c>
+      <c r="C909" t="s">
+        <v>26</v>
+      </c>
+      <c r="D909" t="s">
+        <v>314</v>
+      </c>
+      <c r="E909" t="s">
+        <v>295</v>
+      </c>
+      <c r="F909">
+        <v>0</v>
+      </c>
+      <c r="G909">
+        <v>3.65</v>
+      </c>
+      <c r="H909">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="910" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A910" t="s">
+        <v>29</v>
+      </c>
+      <c r="B910" t="s">
+        <v>30</v>
+      </c>
+      <c r="C910" t="s">
+        <v>10</v>
+      </c>
+      <c r="D910" t="s">
+        <v>27</v>
+      </c>
+      <c r="E910" t="s">
+        <v>28</v>
+      </c>
+      <c r="F910">
+        <v>3</v>
+      </c>
+      <c r="G910">
+        <v>3.75</v>
+      </c>
+      <c r="H910">
+        <v>4048</v>
+      </c>
+    </row>
+    <row r="911" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A911" t="s">
+        <v>8</v>
+      </c>
+      <c r="B911" t="s">
+        <v>9</v>
+      </c>
+      <c r="C911" t="s">
+        <v>19</v>
+      </c>
+      <c r="D911" t="s">
+        <v>173</v>
+      </c>
+      <c r="E911" t="s">
+        <v>24</v>
+      </c>
+      <c r="F911">
+        <v>8</v>
+      </c>
+      <c r="G911">
+        <v>4.07</v>
+      </c>
+      <c r="H911">
+        <v>2432</v>
+      </c>
+    </row>
+    <row r="912" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A912" t="s">
+        <v>13</v>
+      </c>
+      <c r="B912" t="s">
+        <v>14</v>
+      </c>
+      <c r="C912" t="s">
+        <v>15</v>
+      </c>
+      <c r="D912" t="s">
+        <v>360</v>
+      </c>
+      <c r="E912" t="s">
+        <v>136</v>
+      </c>
+      <c r="F912">
+        <v>3</v>
+      </c>
+      <c r="G912">
+        <v>4.2</v>
+      </c>
+      <c r="H912">
+        <v>1496</v>
+      </c>
+    </row>
+    <row r="913" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A913" t="s">
+        <v>17</v>
+      </c>
+      <c r="B913" t="s">
+        <v>18</v>
+      </c>
+      <c r="C913" t="s">
+        <v>26</v>
+      </c>
+      <c r="D913" t="s">
+        <v>104</v>
+      </c>
+      <c r="E913" t="s">
+        <v>104</v>
+      </c>
+      <c r="F913">
+        <v>-3</v>
+      </c>
+      <c r="G913">
+        <v>3.43</v>
+      </c>
+      <c r="H913">
+        <v>3475</v>
+      </c>
+    </row>
+    <row r="914" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A914" t="s">
+        <v>17</v>
+      </c>
+      <c r="B914" t="s">
+        <v>18</v>
+      </c>
+      <c r="C914" t="s">
+        <v>15</v>
+      </c>
+      <c r="D914" t="s">
+        <v>100</v>
+      </c>
+      <c r="E914" t="s">
+        <v>100</v>
+      </c>
+      <c r="F914">
+        <v>-1</v>
+      </c>
+      <c r="G914">
+        <v>4.55</v>
+      </c>
+      <c r="H914">
+        <v>2462</v>
+      </c>
+    </row>
+    <row r="915" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A915" t="s">
+        <v>29</v>
+      </c>
+      <c r="B915" t="s">
+        <v>30</v>
+      </c>
+      <c r="C915" t="s">
+        <v>19</v>
+      </c>
+      <c r="D915" t="s">
+        <v>244</v>
+      </c>
+      <c r="E915" t="s">
+        <v>220</v>
+      </c>
+      <c r="F915">
+        <v>3</v>
+      </c>
+      <c r="G915">
+        <v>3.84</v>
+      </c>
+      <c r="H915">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="916" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A916" t="s">
+        <v>8</v>
+      </c>
+      <c r="B916" t="s">
+        <v>9</v>
+      </c>
+      <c r="C916" t="s">
+        <v>31</v>
+      </c>
+      <c r="D916" t="s">
+        <v>116</v>
+      </c>
+      <c r="E916" t="s">
+        <v>116</v>
+      </c>
+      <c r="F916">
+        <v>-2</v>
+      </c>
+      <c r="G916">
+        <v>3.98</v>
+      </c>
+      <c r="H916">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="917" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A917" t="s">
+        <v>8</v>
+      </c>
+      <c r="B917" t="s">
+        <v>9</v>
+      </c>
+      <c r="C917" t="s">
+        <v>15</v>
+      </c>
+      <c r="D917" t="s">
+        <v>283</v>
+      </c>
+      <c r="E917" t="s">
+        <v>139</v>
+      </c>
+      <c r="F917">
+        <v>1</v>
+      </c>
+      <c r="G917">
+        <v>4.13</v>
+      </c>
+      <c r="H917">
+        <v>3616</v>
+      </c>
+    </row>
+    <row r="918" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A918" t="s">
+        <v>13</v>
+      </c>
+      <c r="B918" t="s">
+        <v>14</v>
+      </c>
+      <c r="C918" t="s">
+        <v>19</v>
+      </c>
+      <c r="D918" t="s">
+        <v>332</v>
+      </c>
+      <c r="E918" t="s">
+        <v>245</v>
+      </c>
+      <c r="F918">
+        <v>1</v>
+      </c>
+      <c r="G918">
+        <v>3.73</v>
+      </c>
+      <c r="H918">
+        <v>3989</v>
+      </c>
+    </row>
+    <row r="919" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A919" t="s">
+        <v>17</v>
+      </c>
+      <c r="B919" t="s">
+        <v>18</v>
+      </c>
+      <c r="C919" t="s">
+        <v>19</v>
+      </c>
+      <c r="D919" t="s">
+        <v>306</v>
+      </c>
+      <c r="E919" t="s">
+        <v>291</v>
+      </c>
+      <c r="F919">
+        <v>1</v>
+      </c>
+      <c r="G919">
+        <v>3.35</v>
+      </c>
+      <c r="H919">
+        <v>4212</v>
+      </c>
+    </row>
+    <row r="920" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A920" t="s">
+        <v>17</v>
+      </c>
+      <c r="B920" t="s">
+        <v>18</v>
+      </c>
+      <c r="C920" t="s">
+        <v>15</v>
+      </c>
+      <c r="D920" t="s">
+        <v>339</v>
+      </c>
+      <c r="E920" t="s">
+        <v>339</v>
+      </c>
+      <c r="F920">
+        <v>1</v>
+      </c>
+      <c r="G920">
+        <v>3.41</v>
+      </c>
+      <c r="H920">
+        <v>3264</v>
+      </c>
+    </row>
+    <row r="921" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A921" t="s">
+        <v>8</v>
+      </c>
+      <c r="B921" t="s">
+        <v>9</v>
+      </c>
+      <c r="C921" t="s">
+        <v>19</v>
+      </c>
+      <c r="D921" t="s">
+        <v>354</v>
+      </c>
+      <c r="E921" t="s">
+        <v>336</v>
+      </c>
+      <c r="F921">
+        <v>6</v>
+      </c>
+      <c r="G921">
+        <v>3.14</v>
+      </c>
+      <c r="H921">
+        <v>1631</v>
+      </c>
+    </row>
+    <row r="922" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A922" t="s">
+        <v>8</v>
+      </c>
+      <c r="C922" t="s">
+        <v>36</v>
+      </c>
+      <c r="D922" t="s">
+        <v>284</v>
+      </c>
+      <c r="E922" t="s">
+        <v>285</v>
+      </c>
+      <c r="F922">
+        <v>-1</v>
+      </c>
+      <c r="G922">
+        <v>3.52</v>
+      </c>
+      <c r="H922">
+        <v>4908</v>
+      </c>
+    </row>
+    <row r="923" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A923" t="s">
+        <v>8</v>
+      </c>
+      <c r="B923" t="s">
+        <v>9</v>
+      </c>
+      <c r="C923" t="s">
+        <v>10</v>
+      </c>
+      <c r="D923" t="s">
+        <v>301</v>
+      </c>
+      <c r="E923" t="s">
+        <v>93</v>
+      </c>
+      <c r="F923">
+        <v>3</v>
+      </c>
+      <c r="G923">
+        <v>3.23</v>
+      </c>
+      <c r="H923">
+        <v>4325</v>
+      </c>
+    </row>
+    <row r="924" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A924" t="s">
+        <v>13</v>
+      </c>
+      <c r="B924" t="s">
+        <v>14</v>
+      </c>
+      <c r="C924" t="s">
+        <v>36</v>
+      </c>
+      <c r="D924" t="s">
+        <v>187</v>
+      </c>
+      <c r="E924" t="s">
+        <v>118</v>
+      </c>
+      <c r="F924">
+        <v>4</v>
+      </c>
+      <c r="G924">
+        <v>6</v>
+      </c>
+      <c r="H924">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="925" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A925" t="s">
+        <v>29</v>
+      </c>
+      <c r="B925" t="s">
+        <v>30</v>
+      </c>
+      <c r="C925" t="s">
+        <v>26</v>
+      </c>
+      <c r="D925" t="s">
+        <v>119</v>
+      </c>
+      <c r="E925" t="s">
+        <v>69</v>
+      </c>
+      <c r="F925">
+        <v>3</v>
+      </c>
+      <c r="G925">
+        <v>3.2</v>
+      </c>
+      <c r="H925">
+        <v>2038</v>
+      </c>
+    </row>
+    <row r="926" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A926" t="s">
+        <v>17</v>
+      </c>
+      <c r="B926" t="s">
+        <v>18</v>
+      </c>
+      <c r="C926" t="s">
+        <v>31</v>
+      </c>
+      <c r="D926" t="s">
+        <v>59</v>
+      </c>
+      <c r="E926" t="s">
+        <v>59</v>
+      </c>
+      <c r="F926">
+        <v>-2</v>
+      </c>
+      <c r="G926">
+        <v>4.8</v>
+      </c>
+      <c r="H926">
+        <v>4231</v>
+      </c>
+    </row>
+    <row r="927" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B927" t="s">
+        <v>14</v>
+      </c>
+      <c r="C927" t="s">
+        <v>36</v>
+      </c>
+      <c r="E927" t="s">
+        <v>48</v>
+      </c>
+      <c r="F927">
+        <v>3</v>
+      </c>
+      <c r="H927">
+        <v>3360</v>
+      </c>
+    </row>
+    <row r="928" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A928" t="s">
+        <v>8</v>
+      </c>
+      <c r="B928" t="s">
+        <v>9</v>
+      </c>
+      <c r="C928" t="s">
+        <v>31</v>
+      </c>
+      <c r="D928" t="s">
+        <v>40</v>
+      </c>
+      <c r="E928" t="s">
+        <v>40</v>
+      </c>
+      <c r="F928">
+        <v>-3</v>
+      </c>
+      <c r="G928">
+        <v>4.68</v>
+      </c>
+      <c r="H928">
+        <v>2540</v>
+      </c>
+    </row>
+    <row r="929" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A929" t="s">
+        <v>13</v>
+      </c>
+      <c r="B929" t="s">
+        <v>14</v>
+      </c>
+      <c r="C929" t="s">
+        <v>36</v>
+      </c>
+      <c r="D929" t="s">
+        <v>41</v>
+      </c>
+      <c r="E929" t="s">
+        <v>96</v>
+      </c>
+      <c r="F929">
+        <v>4</v>
+      </c>
+      <c r="G929">
+        <v>3.49</v>
+      </c>
+      <c r="H929">
+        <v>1733</v>
+      </c>
+    </row>
+    <row r="930" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A930" t="s">
+        <v>13</v>
+      </c>
+      <c r="B930" t="s">
+        <v>14</v>
+      </c>
+      <c r="C930" t="s">
+        <v>15</v>
+      </c>
+      <c r="D930" t="s">
+        <v>213</v>
+      </c>
+      <c r="E930" t="s">
+        <v>352</v>
+      </c>
+      <c r="F930">
+        <v>8</v>
+      </c>
+      <c r="G930">
+        <v>4.8099999999999996</v>
+      </c>
+      <c r="H930">
+        <v>3080</v>
+      </c>
+    </row>
+    <row r="931" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A931" t="s">
+        <v>29</v>
+      </c>
+      <c r="B931" t="s">
+        <v>30</v>
+      </c>
+      <c r="C931" t="s">
+        <v>19</v>
+      </c>
+      <c r="D931" t="s">
+        <v>331</v>
+      </c>
+      <c r="E931" t="s">
+        <v>69</v>
+      </c>
+      <c r="F931">
+        <v>4</v>
+      </c>
+      <c r="G931">
+        <v>4</v>
+      </c>
+      <c r="H931">
+        <v>3298</v>
+      </c>
+    </row>
+    <row r="932" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A932" t="s">
+        <v>29</v>
+      </c>
+      <c r="B932" t="s">
+        <v>30</v>
+      </c>
+      <c r="C932" t="s">
+        <v>10</v>
+      </c>
+      <c r="D932" t="s">
+        <v>93</v>
+      </c>
+      <c r="E932" t="s">
+        <v>263</v>
+      </c>
+      <c r="F932">
+        <v>7</v>
+      </c>
+      <c r="G932">
+        <v>4.0599999999999996</v>
+      </c>
+      <c r="H932">
+        <v>4266</v>
+      </c>
+    </row>
+    <row r="933" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A933" t="s">
+        <v>17</v>
+      </c>
+      <c r="B933" t="s">
+        <v>18</v>
+      </c>
+      <c r="C933" t="s">
+        <v>26</v>
+      </c>
+      <c r="D933" t="s">
+        <v>273</v>
+      </c>
+      <c r="E933" t="s">
+        <v>273</v>
+      </c>
+      <c r="F933">
+        <v>1</v>
+      </c>
+      <c r="G933">
+        <v>3.26</v>
+      </c>
+      <c r="H933">
+        <v>1607</v>
+      </c>
+    </row>
+    <row r="934" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A934" t="s">
+        <v>17</v>
+      </c>
+      <c r="B934" t="s">
+        <v>18</v>
+      </c>
+      <c r="C934" t="s">
+        <v>36</v>
+      </c>
+      <c r="D934" t="s">
+        <v>108</v>
+      </c>
+      <c r="E934" t="s">
+        <v>109</v>
+      </c>
+      <c r="F934">
+        <v>7</v>
+      </c>
+      <c r="G934">
+        <v>3.6</v>
+      </c>
+      <c r="H934">
+        <v>2385</v>
+      </c>
+    </row>
+    <row r="935" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A935" t="s">
+        <v>13</v>
+      </c>
+      <c r="B935" t="s">
+        <v>14</v>
+      </c>
+      <c r="C935" t="s">
+        <v>19</v>
+      </c>
+      <c r="D935" t="s">
+        <v>331</v>
+      </c>
+      <c r="E935" t="s">
+        <v>328</v>
+      </c>
+      <c r="F935">
+        <v>6</v>
+      </c>
+      <c r="G935">
+        <v>4.5199999999999996</v>
+      </c>
+      <c r="H935">
+        <v>3573</v>
+      </c>
+    </row>
+    <row r="936" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A936" t="s">
+        <v>8</v>
+      </c>
+      <c r="B936" t="s">
+        <v>9</v>
+      </c>
+      <c r="C936" t="s">
+        <v>26</v>
+      </c>
+      <c r="D936" t="s">
+        <v>104</v>
+      </c>
+      <c r="E936" t="s">
+        <v>43</v>
+      </c>
+      <c r="F936">
+        <v>0</v>
+      </c>
+      <c r="G936">
+        <v>4.0199999999999996</v>
+      </c>
+      <c r="H936">
+        <v>4936</v>
+      </c>
+    </row>
+    <row r="937" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A937" t="s">
+        <v>17</v>
+      </c>
+      <c r="C937" t="s">
+        <v>31</v>
+      </c>
+      <c r="D937" t="s">
+        <v>280</v>
+      </c>
+      <c r="E937" t="s">
+        <v>283</v>
+      </c>
+      <c r="F937">
+        <v>6</v>
+      </c>
+      <c r="G937">
+        <v>3.58</v>
+      </c>
+      <c r="H937">
+        <v>4168</v>
+      </c>
+    </row>
+    <row r="938" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A938" t="s">
+        <v>8</v>
+      </c>
+      <c r="B938" t="s">
+        <v>9</v>
+      </c>
+      <c r="C938" t="s">
+        <v>36</v>
+      </c>
+      <c r="D938" t="s">
+        <v>146</v>
+      </c>
+      <c r="E938" t="s">
+        <v>350</v>
+      </c>
+      <c r="F938">
+        <v>4</v>
+      </c>
+      <c r="G938">
+        <v>4.59</v>
+      </c>
+      <c r="H938">
+        <v>4486</v>
+      </c>
+    </row>
+    <row r="939" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A939" t="s">
+        <v>29</v>
+      </c>
+      <c r="B939" t="s">
+        <v>30</v>
+      </c>
+      <c r="C939" t="s">
+        <v>19</v>
+      </c>
+      <c r="D939" t="s">
+        <v>96</v>
+      </c>
+      <c r="E939" t="s">
+        <v>97</v>
+      </c>
+      <c r="F939">
+        <v>2</v>
+      </c>
+      <c r="G939">
+        <v>3.35</v>
+      </c>
+      <c r="H939">
+        <v>3368</v>
+      </c>
+    </row>
+    <row r="940" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A940" t="s">
+        <v>29</v>
+      </c>
+      <c r="B940" t="s">
+        <v>30</v>
+      </c>
+      <c r="C940" t="s">
+        <v>10</v>
+      </c>
+      <c r="D940" t="s">
+        <v>179</v>
+      </c>
+      <c r="E940" t="s">
+        <v>179</v>
+      </c>
+      <c r="F940">
+        <v>0</v>
+      </c>
+      <c r="G940">
+        <v>3.99</v>
+      </c>
+      <c r="H940">
+        <v>2730</v>
+      </c>
+    </row>
+    <row r="941" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A941" t="s">
+        <v>17</v>
+      </c>
+      <c r="B941" t="s">
+        <v>18</v>
+      </c>
+      <c r="C941" t="s">
+        <v>26</v>
+      </c>
+      <c r="D941" t="s">
+        <v>50</v>
+      </c>
+      <c r="E941" t="s">
+        <v>101</v>
+      </c>
+      <c r="F941">
+        <v>4</v>
+      </c>
+      <c r="G941">
+        <v>3.42</v>
+      </c>
+      <c r="H941">
+        <v>1870</v>
+      </c>
+    </row>
+    <row r="942" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A942" t="s">
+        <v>13</v>
+      </c>
+      <c r="B942" t="s">
+        <v>14</v>
+      </c>
+      <c r="C942" t="s">
+        <v>15</v>
+      </c>
+      <c r="D942" t="s">
+        <v>43</v>
+      </c>
+      <c r="E942" t="s">
+        <v>44</v>
+      </c>
+      <c r="F942">
+        <v>-1</v>
+      </c>
+      <c r="G942">
+        <v>5.04</v>
+      </c>
+      <c r="H942">
+        <v>3234</v>
+      </c>
+    </row>
+    <row r="943" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A943" t="s">
+        <v>13</v>
+      </c>
+      <c r="B943" t="s">
+        <v>14</v>
+      </c>
+      <c r="C943" t="s">
+        <v>10</v>
+      </c>
+      <c r="D943" t="s">
+        <v>196</v>
+      </c>
+      <c r="E943" t="s">
+        <v>196</v>
+      </c>
+      <c r="F943">
+        <v>2</v>
+      </c>
+      <c r="G943">
+        <v>4.58</v>
+      </c>
+      <c r="H943">
+        <v>4438</v>
+      </c>
+    </row>
+    <row r="944" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A944" t="s">
+        <v>13</v>
+      </c>
+      <c r="B944" t="s">
+        <v>14</v>
+      </c>
+      <c r="C944" t="s">
+        <v>15</v>
+      </c>
+      <c r="D944" t="s">
+        <v>90</v>
+      </c>
+      <c r="E944" t="s">
+        <v>91</v>
+      </c>
+      <c r="F944">
+        <v>5</v>
+      </c>
+      <c r="G944">
+        <v>2.88</v>
+      </c>
+      <c r="H944">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="945" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A945" t="s">
+        <v>29</v>
+      </c>
+      <c r="B945" t="s">
+        <v>30</v>
+      </c>
+      <c r="C945" t="s">
+        <v>10</v>
+      </c>
+      <c r="D945" t="s">
+        <v>160</v>
+      </c>
+      <c r="E945" t="s">
+        <v>109</v>
+      </c>
+      <c r="F945">
+        <v>8</v>
+      </c>
+      <c r="G945">
+        <v>3.65</v>
+      </c>
+      <c r="H945">
+        <v>1901</v>
+      </c>
+    </row>
+    <row r="946" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A946" t="s">
+        <v>13</v>
+      </c>
+      <c r="B946" t="s">
+        <v>14</v>
+      </c>
+      <c r="C946" t="s">
+        <v>36</v>
+      </c>
+      <c r="D946" t="s">
+        <v>193</v>
+      </c>
+      <c r="E946" t="s">
+        <v>158</v>
+      </c>
+      <c r="F946">
+        <v>6</v>
+      </c>
+      <c r="G946">
+        <v>2</v>
+      </c>
+      <c r="H946">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="947" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A947" t="s">
+        <v>17</v>
+      </c>
+      <c r="B947" t="s">
+        <v>18</v>
+      </c>
+      <c r="C947" t="s">
+        <v>36</v>
+      </c>
+      <c r="D947" t="s">
+        <v>291</v>
+      </c>
+      <c r="E947" t="s">
+        <v>32</v>
+      </c>
+      <c r="F947">
+        <v>7</v>
+      </c>
+      <c r="G947">
+        <v>3.01</v>
+      </c>
+      <c r="H947">
+        <v>2194</v>
+      </c>
+    </row>
+    <row r="948" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A948" t="s">
+        <v>8</v>
+      </c>
+      <c r="B948" t="s">
+        <v>9</v>
+      </c>
+      <c r="C948" t="s">
+        <v>31</v>
+      </c>
+      <c r="D948" t="s">
+        <v>241</v>
+      </c>
+      <c r="E948" t="s">
+        <v>163</v>
+      </c>
+      <c r="F948">
+        <v>2</v>
+      </c>
+      <c r="G948">
+        <v>4.6399999999999997</v>
+      </c>
+      <c r="H948">
+        <v>1778</v>
+      </c>
+    </row>
+    <row r="949" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A949" t="s">
+        <v>8</v>
+      </c>
+      <c r="B949" t="s">
+        <v>9</v>
+      </c>
+      <c r="C949" t="s">
+        <v>36</v>
+      </c>
+      <c r="D949" t="s">
+        <v>210</v>
+      </c>
+      <c r="E949" t="s">
+        <v>267</v>
+      </c>
+      <c r="F949">
+        <v>-1</v>
+      </c>
+      <c r="G949">
+        <v>3.76</v>
+      </c>
+      <c r="H949">
+        <v>2533</v>
+      </c>
+    </row>
+    <row r="950" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A950" t="s">
+        <v>8</v>
+      </c>
+      <c r="B950" t="s">
+        <v>9</v>
+      </c>
+      <c r="C950" t="s">
+        <v>26</v>
+      </c>
+      <c r="D950" t="s">
+        <v>292</v>
+      </c>
+      <c r="E950" t="s">
+        <v>264</v>
+      </c>
+      <c r="F950">
+        <v>4</v>
+      </c>
+      <c r="G950">
+        <v>4.2</v>
+      </c>
+      <c r="H950">
+        <v>3470</v>
+      </c>
+    </row>
+    <row r="951" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A951" t="s">
+        <v>13</v>
+      </c>
+      <c r="B951" t="s">
+        <v>14</v>
+      </c>
+      <c r="C951" t="s">
+        <v>26</v>
+      </c>
+      <c r="D951" t="s">
+        <v>123</v>
+      </c>
+      <c r="E951" t="s">
+        <v>56</v>
+      </c>
+      <c r="F951">
+        <v>4</v>
+      </c>
+      <c r="G951">
+        <v>3.6</v>
+      </c>
+      <c r="H951">
+        <v>4909</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>